<commit_message>
🤖 Deploy E2E Master QA Portal: Build #2 ae4e6b4fe0f710fcec1bc9c9b9ba10a61d9fb1e7
</commit_message>
<xml_diff>
--- a/Master_Automation_Report.xlsx
+++ b/Master_Automation_Report.xlsx
@@ -459,7 +459,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -483,7 +483,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-23 05:47:38</t>
+          <t>2026-07-23 05:54:21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
🤖 Deploy E2E Master QA Portal: Build #4 590d17aa91afa3e000adf76ff0e9f655cc946a67
</commit_message>
<xml_diff>
--- a/Master_Automation_Report.xlsx
+++ b/Master_Automation_Report.xlsx
@@ -459,7 +459,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -483,7 +483,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-07-23 06:03:05</t>
+          <t>2026-07-23 06:09:30</t>
         </is>
       </c>
     </row>
@@ -554,7 +554,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>SELENIUM</t>
+          <t>TC_SEL</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -577,7 +577,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>APPIUM</t>
+          <t>TC_APP</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -600,7 +600,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>UNIT</t>
+          <t>TC_UNI</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -623,7 +623,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>VALIDATION</t>
+          <t>TC_VAL</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -646,7 +646,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DEPLOYMENT</t>
+          <t>TC_DEP</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -669,7 +669,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PERFORMANCE</t>
+          <t>TC_PERF</t>
         </is>
       </c>
       <c r="C16" t="n">

</xml_diff>